<commit_message>
apply FX conversion to Market-to-Book and MVA
</commit_message>
<xml_diff>
--- a/models/builds/2026-05-14-luong-iqiyi-financials.xlsx
+++ b/models/builds/2026-05-14-luong-iqiyi-financials.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luongduyphuong/Documents/GitHub/Corporate-Finance/models/builds/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4E33CD7-4A07-5F44-B77D-00CC3667660B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62DD2FB6-05A4-304A-893A-DECC8D95A672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,9 +21,9 @@
     <sheet name="Notes" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="avg_equity">Ratios!$C$36</definedName>
-    <definedName name="avg_total_assets">Ratios!$C$37</definedName>
-    <definedName name="avg_total_capitalization">Ratios!$C$38</definedName>
+    <definedName name="avg_equity">Ratios!$C$37</definedName>
+    <definedName name="avg_total_assets">Ratios!$C$38</definedName>
+    <definedName name="avg_total_capitalization">Ratios!$C$39</definedName>
     <definedName name="BAL_accounts_payable_curr">'Balance Sheet'!$G$8</definedName>
     <definedName name="BAL_accounts_payable_prior">'Balance Sheet'!$H$8</definedName>
     <definedName name="BAL_accumulated_depreciation_curr">'Balance Sheet'!$C$15</definedName>
@@ -70,18 +70,19 @@
     <definedName name="CASH_operating">'Cash Flow Statement'!$C$17</definedName>
     <definedName name="CF_depreciation_amortization">'Cash Flow Statement'!$C$8</definedName>
     <definedName name="cost_capital">Ratios!$C$10</definedName>
-    <definedName name="currentYear_after_tax_operating_income">Ratios!$C$22</definedName>
-    <definedName name="currentYear_assets_current">Ratios!$C$26</definedName>
-    <definedName name="currentYear_assets_total">Ratios!$C$31</definedName>
-    <definedName name="currentYear_cash_marketable_securities">Ratios!$C$25</definedName>
-    <definedName name="currentYear_cost_goods_sold_daily">Ratios!$C$28</definedName>
-    <definedName name="currentYear_daily_sales_average">Ratios!$C$23</definedName>
-    <definedName name="currentYear_debt_long_term">Ratios!$C$29</definedName>
-    <definedName name="currentYear_equity">Ratios!$C$24</definedName>
-    <definedName name="currentYear_liabilities_current">Ratios!$C$27</definedName>
-    <definedName name="currentYear_liabilities_total">Ratios!$C$33</definedName>
-    <definedName name="currentYear_total_capitalization">Ratios!$C$32</definedName>
-    <definedName name="currentYear_working_capital_net">Ratios!$C$30</definedName>
+    <definedName name="currentYear_after_tax_operating_income">Ratios!$C$23</definedName>
+    <definedName name="currentYear_assets_current">Ratios!$C$27</definedName>
+    <definedName name="currentYear_assets_total">Ratios!$C$32</definedName>
+    <definedName name="currentYear_cash_marketable_securities">Ratios!$C$26</definedName>
+    <definedName name="currentYear_cost_goods_sold_daily">Ratios!$C$29</definedName>
+    <definedName name="currentYear_daily_sales_average">Ratios!$C$24</definedName>
+    <definedName name="currentYear_debt_long_term">Ratios!$C$30</definedName>
+    <definedName name="currentYear_equity">Ratios!$C$25</definedName>
+    <definedName name="currentYear_liabilities_current">Ratios!$C$28</definedName>
+    <definedName name="currentYear_liabilities_total">Ratios!$C$34</definedName>
+    <definedName name="currentYear_total_capitalization">Ratios!$C$33</definedName>
+    <definedName name="currentYear_working_capital_net">Ratios!$C$31</definedName>
+    <definedName name="fx_usd_cny" comment="Dec 31 2025 USD/CNY from 20-F Note 2">Ratios!$C$13</definedName>
     <definedName name="INC_addition_retained_earnings">'Income Statement'!$C$19</definedName>
     <definedName name="INC_cost_goods_sold">'Income Statement'!$C$7</definedName>
     <definedName name="INC_depreciation">'Income Statement'!$C$9</definedName>
@@ -95,17 +96,17 @@
     <definedName name="INC_taxable_income">'Income Statement'!$C$13</definedName>
     <definedName name="INC_taxes">'Income Statement'!$C$14</definedName>
     <definedName name="market_capitalization">Ratios!$C$12</definedName>
-    <definedName name="RATIO_asset_turnover">Ratios!$C$54</definedName>
-    <definedName name="RATIO_debt_burden">Ratios!$C$67</definedName>
-    <definedName name="RATIO_leverage">Ratios!$C$68</definedName>
-    <definedName name="RATIO_operating_profit_margin">Ratios!$C$60</definedName>
+    <definedName name="RATIO_asset_turnover">Ratios!$C$55</definedName>
+    <definedName name="RATIO_debt_burden">Ratios!$C$68</definedName>
+    <definedName name="RATIO_leverage">Ratios!$C$69</definedName>
+    <definedName name="RATIO_operating_profit_margin">Ratios!$C$61</definedName>
     <definedName name="share_price">Ratios!$C$8</definedName>
     <definedName name="shares_outstanding">Ratios!$C$9</definedName>
-    <definedName name="startYear_equity">Ratios!$C$15</definedName>
-    <definedName name="startYear_inventory">Ratios!$C$16</definedName>
-    <definedName name="startYear_receivables">Ratios!$C$17</definedName>
-    <definedName name="startYear_total_assets">Ratios!$C$18</definedName>
-    <definedName name="startYear_total_capitalization">Ratios!$C$19</definedName>
+    <definedName name="startYear_equity">Ratios!$C$16</definedName>
+    <definedName name="startYear_inventory">Ratios!$C$17</definedName>
+    <definedName name="startYear_receivables">Ratios!$C$18</definedName>
+    <definedName name="startYear_total_assets">Ratios!$C$19</definedName>
+    <definedName name="startYear_total_capitalization">Ratios!$C$20</definedName>
     <definedName name="tax_rate">Ratios!$C$11</definedName>
     <definedName name="yearCurrent">Ratios!$C$6</definedName>
     <definedName name="yearStart">Ratios!$C$7</definedName>
@@ -172,6 +173,40 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={8C1E391D-7710-314C-AE28-570BA31CB27C}</author>
+    <author>tc={1569627C-8252-D846-96C4-0EAC61EA9C66}</author>
+  </authors>
+  <commentList>
+    <comment ref="C44" authorId="0" shapeId="0" xr:uid="{8C1E391D-7710-314C-AE28-570BA31CB27C}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    FX ADJUSTMENT (20-F Note 2):
+market_capitalization = USD ('000); currentYear_equity = RMB ('000).
+Divide RMB equity by fx_usd_cny (6.9956) → USD before subtracting.
+Source: Form 20-F FY2025, Note 2 — RMB 6.9956 = US$1.00 (Dec 31 2025).</t>
+      </text>
+    </comment>
+    <comment ref="C45" authorId="1" shapeId="0" xr:uid="{1569627C-8252-D846-96C4-0EAC61EA9C66}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    FX ADJUSTMENT (20-F Note 2):
+market_capitalization = USD ('000); currentYear_equity = RMB ('000).
+Divide RMB equity by fx_usd_cny (6.9956) → USD before dividing.
+Corrected P/B = 0.60x  (was 0.085x before FX fix).
+Source: Form 20-F FY2025, Note 2 — RMB 6.9956 = US$1.00 (Dec 31 2025).</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Lương Duy Phương</author>
@@ -527,7 +562,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="354">
   <si>
     <t>Ratios &amp; Derived Inputs</t>
   </si>
@@ -799,13 +834,7 @@
     <t>Market value added (MVA)</t>
   </si>
   <si>
-    <t>market_capitalization − currentYear_equity</t>
-  </si>
-  <si>
     <t>Market-to-book ratio</t>
-  </si>
-  <si>
-    <t>market_capitalization / currentYear_equity</t>
   </si>
   <si>
     <t>Economic value added (EVA)</t>
@@ -1580,13 +1609,31 @@
   </si>
   <si>
     <t>Source: 20-F Cover Page — 'The financial statements are prepared in accordance with US GAAP'</t>
+  </si>
+  <si>
+    <t>fx_usd_cny</t>
+  </si>
+  <si>
+    <t>USD/CNY FX rate (Dec 31, 2025)</t>
+  </si>
+  <si>
+    <t>per 20-F Note 2 (Dec 31 2025 rate)</t>
+  </si>
+  <si>
+    <t>Source: SEC EDGAR Form 20-F FY2025, Note 2 — RMB 6.9956 = US$1.00 (Dec 31, 2025 closing rate). Used to convert RMB equity to USD for MVA &amp; Market-to-Book calculations.</t>
+  </si>
+  <si>
+    <t>market_capitalization − (currentYear_equity / fx_usd_cny)</t>
+  </si>
+  <si>
+    <t>market_capitalization / (currentYear_equity / fx_usd_cny)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);&quot;—&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0%;\(0.0%\);&quot;—&quot;"/>
@@ -1595,8 +1642,9 @@
     <numFmt numFmtId="169" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="170" formatCode="0.0&quot; days&quot;"/>
     <numFmt numFmtId="171" formatCode="0.000"/>
+    <numFmt numFmtId="172" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1741,8 +1789,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF525252"/>
+      <name val="Consolas"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1785,8 +1839,14 @@
         <bgColor rgb="FFE6F2EF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -1809,11 +1869,57 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1869,7 +1975,6 @@
     <xf numFmtId="167" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1899,15 +2004,23 @@
     </xf>
     <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="172" fontId="9" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1923,6 +2036,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Phuong Luong" id="{0B72969E-1948-C942-AE7E-6B52846BA07C}" userId="d3437353e2f3d7aa" providerId="Windows Live"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2208,6 +2327,24 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="C44" dT="2026-05-17T00:50:29.45" personId="{0B72969E-1948-C942-AE7E-6B52846BA07C}" id="{8C1E391D-7710-314C-AE28-570BA31CB27C}">
+    <text>FX ADJUSTMENT (20-F Note 2):
+market_capitalization = USD ('000); currentYear_equity = RMB ('000).
+Divide RMB equity by fx_usd_cny (6.9956) → USD before subtracting.
+Source: Form 20-F FY2025, Note 2 — RMB 6.9956 = US$1.00 (Dec 31 2025).</text>
+  </threadedComment>
+  <threadedComment ref="C45" dT="2026-05-17T00:50:29.46" personId="{0B72969E-1948-C942-AE7E-6B52846BA07C}" id="{1569627C-8252-D846-96C4-0EAC61EA9C66}">
+    <text>FX ADJUSTMENT (20-F Note 2):
+market_capitalization = USD ('000); currentYear_equity = RMB ('000).
+Divide RMB equity by fx_usd_cny (6.9956) → USD before dividing.
+Corrected P/B = 0.60x  (was 0.085x before FX fix).
+Source: Form 20-F FY2025, Note 2 — RMB 6.9956 = US$1.00 (Dec 31 2025).</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
   <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
@@ -2246,22 +2383,22 @@
       <c r="C2" s="1"/>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B4" s="49" t="s">
-        <v>155</v>
-      </c>
-      <c r="C4" s="50"/>
+      <c r="B4" s="50" t="s">
+        <v>153</v>
+      </c>
+      <c r="C4" s="49"/>
     </row>
     <row r="5" spans="2:3" ht="26" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="53" t="s">
-        <v>156</v>
-      </c>
-      <c r="C5" s="50"/>
+        <v>154</v>
+      </c>
+      <c r="C5" s="49"/>
     </row>
     <row r="6" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="51" t="s">
-        <v>157</v>
-      </c>
-      <c r="C6" s="50"/>
+        <v>155</v>
+      </c>
+      <c r="C6" s="49"/>
     </row>
     <row r="7" spans="2:3" ht="4" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="2"/>
@@ -2269,209 +2406,209 @@
     </row>
     <row r="9" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="52" t="s">
-        <v>158</v>
-      </c>
-      <c r="C9" s="50"/>
+        <v>156</v>
+      </c>
+      <c r="C9" s="49"/>
     </row>
     <row r="10" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="14" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="52" t="s">
-        <v>171</v>
-      </c>
-      <c r="C17" s="50"/>
+        <v>169</v>
+      </c>
+      <c r="C17" s="49"/>
     </row>
     <row r="18" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="19" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="6" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="8" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="9" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="22" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="10" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="24" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="52" t="s">
-        <v>182</v>
-      </c>
-      <c r="C24" s="50"/>
+        <v>180</v>
+      </c>
+      <c r="C24" s="49"/>
     </row>
     <row r="25" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="26" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="11" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="27" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="11" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="28" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="11" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="29" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="11" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="30" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="11" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="11" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="32" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="11" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="33" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="11" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="36" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B36" s="52" t="s">
-        <v>200</v>
-      </c>
-      <c r="C36" s="50"/>
+        <v>198</v>
+      </c>
+      <c r="C36" s="49"/>
     </row>
     <row r="37" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="12" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="38" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="12" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B41" s="54" t="s">
-        <v>205</v>
-      </c>
-      <c r="C41" s="50"/>
+        <v>203</v>
+      </c>
+      <c r="C41" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -2503,45 +2640,45 @@
   <sheetData>
     <row r="2" spans="2:8" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="14" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B3" s="15" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="16" t="s">
+        <v>206</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>207</v>
+      </c>
+      <c r="D5" s="17" t="s">
         <v>208</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="F5" s="16" t="s">
         <v>209</v>
       </c>
-      <c r="D5" s="17" t="s">
-        <v>210</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>211</v>
-      </c>
       <c r="G5" s="17" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="18" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="12" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C7" s="19">
         <v>4354275</v>
@@ -2550,7 +2687,7 @@
         <v>3529679</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="G7" s="19">
         <v>4690642</v>
@@ -2561,7 +2698,7 @@
     </row>
     <row r="8" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="12" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C8" s="19">
         <v>2522668</v>
@@ -2570,7 +2707,7 @@
         <v>2191178</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="G8" s="19">
         <v>6652432</v>
@@ -2581,7 +2718,7 @@
     </row>
     <row r="9" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="12" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C9" s="19">
         <v>447507</v>
@@ -2590,7 +2727,7 @@
         <v>388718</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="G9" s="19">
         <v>10724233</v>
@@ -2601,7 +2738,7 @@
     </row>
     <row r="10" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="12" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C10" s="19">
         <v>2965845</v>
@@ -2610,7 +2747,7 @@
         <v>3417661</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="G10" s="21">
         <f>SUM(G7:G9)</f>
@@ -2623,7 +2760,7 @@
     </row>
     <row r="11" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="20" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C11" s="21">
         <f>SUM(C7:C10)</f>
@@ -2647,10 +2784,10 @@
     </row>
     <row r="13" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="18" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="G13" s="19">
         <v>1224678</v>
@@ -2661,7 +2798,7 @@
     </row>
     <row r="14" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="12" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C14" s="19">
         <v>903427</v>
@@ -2672,7 +2809,7 @@
     </row>
     <row r="15" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="12" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C15" s="19">
         <v>0</v>
@@ -2680,11 +2817,11 @@
       <c r="D15" s="19">
         <v>0</v>
       </c>
-      <c r="E15" s="48" t="s">
-        <v>338</v>
+      <c r="E15" s="47" t="s">
+        <v>336</v>
       </c>
       <c r="F15" s="20" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="G15" s="21">
         <f>G10+G12+G13</f>
@@ -2697,7 +2834,7 @@
     </row>
     <row r="16" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="20" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C16" s="21">
         <f>C14-C15</f>
@@ -2707,21 +2844,21 @@
         <f>D14-D15</f>
         <v>877982</v>
       </c>
-      <c r="E16" s="48" t="s">
-        <v>339</v>
+      <c r="E16" s="47" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F17" s="18" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="18" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="G18" s="19">
         <v>56026664</v>
@@ -2732,7 +2869,7 @@
     </row>
     <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="12" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C19" s="19">
         <v>3820823</v>
@@ -2741,7 +2878,7 @@
         <v>3820823</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="G19" s="19">
         <v>-42717738</v>
@@ -2752,7 +2889,7 @@
     </row>
     <row r="20" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="12" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C20" s="19">
         <v>31667190</v>
@@ -2761,7 +2898,7 @@
         <v>31534484</v>
       </c>
       <c r="F20" s="20" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="G20" s="21">
         <f>G18+G19</f>
@@ -2775,7 +2912,7 @@
     <row r="22" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="23" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C23" s="22">
         <f>C11+C16+C19+C20</f>
@@ -2786,7 +2923,7 @@
         <v>45760525</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="G23" s="22">
         <f>G15+G20</f>
@@ -2815,28 +2952,28 @@
   <sheetData>
     <row r="2" spans="2:4" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="14" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" s="15" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>237</v>
+      </c>
+      <c r="D5" s="23" t="s">
         <v>238</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>239</v>
-      </c>
-      <c r="D5" s="23" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="12" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C6" s="19">
         <v>27291300</v>
@@ -2847,7 +2984,7 @@
     </row>
     <row r="7" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="12" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C7" s="19">
         <v>21542347</v>
@@ -2859,7 +2996,7 @@
     </row>
     <row r="8" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="12" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C8" s="19">
         <v>5519638</v>
@@ -2871,7 +3008,7 @@
     </row>
     <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="12" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C9" s="19">
         <v>0</v>
@@ -2883,7 +3020,7 @@
     </row>
     <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="20" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C10" s="21">
         <f>C6-C7-C8-C9</f>
@@ -2896,7 +3033,7 @@
     </row>
     <row r="11" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="12" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C11" s="19">
         <v>620800</v>
@@ -2908,7 +3045,7 @@
     </row>
     <row r="12" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="12" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C12" s="19">
         <v>909616</v>
@@ -2920,7 +3057,7 @@
     </row>
     <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="20" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C13" s="21">
         <f>C10+C11-C12</f>
@@ -2933,7 +3070,7 @@
     </row>
     <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="12" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C14" s="19">
         <v>144542</v>
@@ -2945,7 +3082,7 @@
     </row>
     <row r="15" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C15" s="22">
         <f>C13-C14</f>
@@ -2958,12 +3095,12 @@
     </row>
     <row r="17" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="18" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="12" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C18" s="19">
         <v>0</v>
@@ -2975,7 +3112,7 @@
     </row>
     <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="20" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C19" s="21">
         <f>C15-C18</f>
@@ -3005,129 +3142,129 @@
   <sheetData>
     <row r="2" spans="2:4" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="14" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" s="15" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="23" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="18" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="D6" s="15"/>
     </row>
     <row r="7" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="12" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C7" s="27">
         <f>INC_net</f>
         <v>-204043</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="8" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="12" t="s">
-        <v>259</v>
-      </c>
-      <c r="C8" s="47">
+        <v>257</v>
+      </c>
+      <c r="C8" s="46">
         <v>13264120</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="12" t="s">
-        <v>333</v>
-      </c>
-      <c r="C9" s="47">
+        <v>331</v>
+      </c>
+      <c r="C9" s="46">
         <v>99099</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="28" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="D10" s="15"/>
     </row>
     <row r="11" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="12" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C11" s="19">
         <v>-350341</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="12" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="12" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C12" s="19">
         <v>-4858452</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="12" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C13" s="19">
         <v>-8199131</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="12" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C14" s="19">
         <v>322196</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="12" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C15" s="19">
         <v>32353</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="20" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C16" s="21">
         <f>SUM(C11:C15)</f>
@@ -3137,7 +3274,7 @@
     </row>
     <row r="17" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="5" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C17" s="22">
         <f>C7+C8+C9+C16</f>
@@ -3150,13 +3287,13 @@
     </row>
     <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="18" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D19" s="15"/>
     </row>
     <row r="20" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="12" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C20" s="19">
         <v>-124636</v>
@@ -3165,7 +3302,7 @@
     </row>
     <row r="21" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="12" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C21" s="19">
         <v>721422</v>
@@ -3174,7 +3311,7 @@
     </row>
     <row r="22" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="12" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C22" s="19">
         <v>-924221</v>
@@ -3183,7 +3320,7 @@
     </row>
     <row r="23" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C23" s="22">
         <f>SUM(C20:C22)</f>
@@ -3196,13 +3333,13 @@
     </row>
     <row r="25" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="18" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="D25" s="15"/>
     </row>
     <row r="26" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="12" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C26" s="19">
         <v>-1294246</v>
@@ -3211,7 +3348,7 @@
     </row>
     <row r="27" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="12" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C27" s="19">
         <v>2578911</v>
@@ -3220,7 +3357,7 @@
     </row>
     <row r="28" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="12" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C28" s="19">
         <v>-19455</v>
@@ -3229,7 +3366,7 @@
     </row>
     <row r="29" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="12" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C29" s="19">
         <v>347</v>
@@ -3238,7 +3375,7 @@
     </row>
     <row r="30" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="12" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C30" s="19">
         <v>-201123</v>
@@ -3247,7 +3384,7 @@
     </row>
     <row r="31" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="5" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C31" s="22">
         <f>SUM(C26:C30)</f>
@@ -3257,16 +3394,16 @@
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B32" s="12" t="s">
-        <v>319</v>
-      </c>
-      <c r="C32" s="45">
+        <v>317</v>
+      </c>
+      <c r="C32" s="44">
         <v>-55393</v>
       </c>
       <c r="D32" s="15"/>
     </row>
     <row r="33" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C33" s="22">
         <f>C17+C23+C31+C32</f>
@@ -3280,8 +3417,8 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="B2:F76"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="B2:F77"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -3357,7 +3494,7 @@
     </row>
     <row r="9" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="12" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C9" s="33">
         <v>962959</v>
@@ -3366,8 +3503,8 @@
       <c r="E9" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="48" t="s">
-        <v>341</v>
+      <c r="F9" s="47" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -3398,7 +3535,7 @@
       <c r="B12" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="35">
+      <c r="C12" s="56">
         <f>share_price*shares_outstanding</f>
         <v>1136291.6199999999</v>
       </c>
@@ -3409,793 +3546,811 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="55" t="s">
+    <row r="13" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="55" t="s">
+        <v>349</v>
+      </c>
+      <c r="C13" s="60">
+        <v>6.9955999999999996</v>
+      </c>
+      <c r="D13" s="58" t="s">
+        <v>350</v>
+      </c>
+      <c r="E13" s="57" t="s">
+        <v>348</v>
+      </c>
+      <c r="F13" s="59" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="50"/>
-      <c r="D14" s="50"/>
-      <c r="E14" s="50"/>
-    </row>
-    <row r="15" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="12" t="s">
+      <c r="C15" s="49"/>
+      <c r="D15" s="49"/>
+      <c r="E15" s="49"/>
+    </row>
+    <row r="16" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="36">
+      <c r="C16" s="35">
         <f>BAL_equity_shareholders_prior</f>
         <v>13373764</v>
       </c>
-      <c r="D15" s="30" t="s">
+      <c r="D16" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="E15" s="30" t="s">
+      <c r="E16" s="30" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="12" t="s">
+    <row r="17" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="36">
+      <c r="C17" s="35">
         <f>BAL_inventories_prior</f>
         <v>388718</v>
       </c>
-      <c r="D16" s="30" t="s">
+      <c r="D17" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="E16" s="30" t="s">
+      <c r="E17" s="30" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="12" t="s">
+    <row r="18" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="36">
+      <c r="C18" s="35">
         <f>BAL_receivables_prior</f>
         <v>2191178</v>
       </c>
-      <c r="D17" s="30" t="s">
+      <c r="D18" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="E17" s="30" t="s">
+      <c r="E18" s="30" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="12" t="s">
+    <row r="19" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="36">
+      <c r="C19" s="35">
         <f>BAL_assets_total_prior</f>
         <v>45760525</v>
       </c>
-      <c r="D18" s="30" t="s">
+      <c r="D19" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="E18" s="30" t="s">
+      <c r="E19" s="30" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="12" t="s">
+    <row r="20" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="C19" s="36">
+      <c r="C20" s="35">
         <f>BAL_debt_long_term_prior+BAL_equity_shareholders_prior</f>
         <v>22761169</v>
       </c>
-      <c r="D19" s="30" t="s">
+      <c r="D20" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="E19" s="30" t="s">
+      <c r="E20" s="30" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="55" t="s">
+    <row r="22" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="C21" s="50"/>
-      <c r="D21" s="50"/>
-      <c r="E21" s="50"/>
-    </row>
-    <row r="22" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="12" t="s">
+      <c r="C22" s="49"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="49"/>
+    </row>
+    <row r="23" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C22" s="36">
+      <c r="C23" s="35">
         <f>INC_net+(1-tax_rate)*INC_interest_expense</f>
         <v>478169</v>
       </c>
-      <c r="D22" s="30" t="s">
+      <c r="D23" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="E22" s="30" t="s">
+      <c r="E23" s="30" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="12" t="s">
+    <row r="24" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="C23" s="37">
+      <c r="C24" s="36">
         <f>IFERROR(INC_sales/365,"")</f>
         <v>74770.684931506854</v>
       </c>
-      <c r="D23" s="30" t="s">
+      <c r="D24" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="E23" s="30" t="s">
+      <c r="E24" s="30" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="24" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="12" t="s">
+    <row r="25" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="C24" s="36">
+      <c r="C25" s="35">
         <f>BAL_equity_shareholders_curr</f>
         <v>13308926</v>
       </c>
-      <c r="D24" s="30" t="s">
+      <c r="D25" s="30" t="s">
         <v>45</v>
       </c>
-      <c r="E24" s="30" t="s">
+      <c r="E25" s="30" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="12" t="s">
+    <row r="26" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B26" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="C25" s="36">
+      <c r="C26" s="35">
         <f>BAL_cash_marketable_securities_curr</f>
         <v>4354275</v>
       </c>
-      <c r="D25" s="30" t="s">
+      <c r="D26" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="E25" s="30" t="s">
+      <c r="E26" s="30" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="12" t="s">
+    <row r="27" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B27" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="C26" s="36">
+      <c r="C27" s="35">
         <f>BAL_assets_current_curr</f>
         <v>10290295</v>
       </c>
-      <c r="D26" s="30" t="s">
+      <c r="D27" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="E26" s="30" t="s">
+      <c r="E27" s="30" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="27" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="12" t="s">
+    <row r="28" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B28" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="C27" s="36">
+      <c r="C28" s="35">
         <f>BAL_liabilities_current_curr</f>
         <v>22067307</v>
       </c>
-      <c r="D27" s="30" t="s">
+      <c r="D28" s="30" t="s">
         <v>54</v>
       </c>
-      <c r="E27" s="30" t="s">
+      <c r="E28" s="30" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="28" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="12" t="s">
+    <row r="29" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B29" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C28" s="37">
+      <c r="C29" s="36">
         <f>IFERROR(INC_cost_goods_sold/365,"")</f>
         <v>59020.128767123286</v>
       </c>
-      <c r="D28" s="30" t="s">
+      <c r="D29" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="E28" s="30" t="s">
+      <c r="E29" s="30" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="29" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="12" t="s">
+    <row r="30" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B30" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="C29" s="36">
+      <c r="C30" s="35">
         <f>BAL_debt_long_term_curr</f>
         <v>10080824</v>
       </c>
-      <c r="D29" s="30" t="s">
+      <c r="D30" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="E29" s="30" t="s">
+      <c r="E30" s="30" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="30" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="12" t="s">
+    <row r="31" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B31" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="C30" s="36">
+      <c r="C31" s="35">
         <f>BAL_assets_current_curr-BAL_liabilities_current_curr</f>
         <v>-11777012</v>
       </c>
-      <c r="D30" s="30" t="s">
+      <c r="D31" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="E30" s="30" t="s">
+      <c r="E31" s="30" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="31" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="12" t="s">
+    <row r="32" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B32" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="C31" s="36">
+      <c r="C32" s="35">
         <f>BAL_assets_total_curr</f>
         <v>46681735</v>
       </c>
-      <c r="D31" s="30" t="s">
+      <c r="D32" s="30" t="s">
         <v>66</v>
       </c>
-      <c r="E31" s="30" t="s">
+      <c r="E32" s="30" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="32" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="12" t="s">
+    <row r="33" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B33" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="C32" s="36">
+      <c r="C33" s="35">
         <f>BAL_debt_long_term_curr+BAL_equity_shareholders_curr</f>
         <v>23389750</v>
       </c>
-      <c r="D32" s="30" t="s">
+      <c r="D33" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="E32" s="30" t="s">
+      <c r="E33" s="30" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="33" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="12" t="s">
+    <row r="34" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B34" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C33" s="36">
+      <c r="C34" s="35">
         <f>BAL_liabilities_total_curr</f>
         <v>33372809</v>
       </c>
-      <c r="D33" s="30" t="s">
+      <c r="D34" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="E33" s="30" t="s">
+      <c r="E34" s="30" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="35" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="55" t="s">
+    <row r="36" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B36" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="C35" s="50"/>
-      <c r="D35" s="50"/>
-      <c r="E35" s="50"/>
-    </row>
-    <row r="36" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="12" t="s">
+      <c r="C36" s="49"/>
+      <c r="D36" s="49"/>
+      <c r="E36" s="49"/>
+    </row>
+    <row r="37" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B37" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="C36" s="37">
+      <c r="C37" s="36">
         <f>AVERAGE(startYear_equity,currentYear_equity)</f>
         <v>13341345</v>
       </c>
-      <c r="D36" s="30" t="s">
+      <c r="D37" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="E36" s="30" t="s">
+      <c r="E37" s="30" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="37" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="12" t="s">
+    <row r="38" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B38" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="C37" s="37">
+      <c r="C38" s="36">
         <f>AVERAGE(startYear_total_assets,currentYear_assets_total)</f>
         <v>46221130</v>
       </c>
-      <c r="D37" s="30" t="s">
+      <c r="D38" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="E37" s="30" t="s">
+      <c r="E38" s="30" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="38" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="12" t="s">
+    <row r="39" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B39" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="C38" s="37">
+      <c r="C39" s="36">
         <f>AVERAGE(startYear_total_capitalization,currentYear_total_capitalization)</f>
         <v>23075459.5</v>
       </c>
-      <c r="D38" s="30" t="s">
+      <c r="D39" s="30" t="s">
         <v>82</v>
       </c>
-      <c r="E38" s="30" t="s">
+      <c r="E39" s="30" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="41" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B41" s="23" t="s">
+    <row r="42" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B42" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="C41" s="23" t="s">
+      <c r="C42" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="D41" s="23" t="s">
+      <c r="D42" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="E41" s="23" t="s">
+      <c r="E42" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="F41" s="23" t="s">
+      <c r="F42" s="23" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="42" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="5" t="s">
+    <row r="43" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B43" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="C42" s="1"/>
-      <c r="D42" s="1"/>
-      <c r="E42" s="1"/>
-    </row>
-    <row r="43" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B43" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="C43" s="38">
-        <f>market_capitalization - currentYear_equity</f>
-        <v>-12172634.380000001</v>
-      </c>
-      <c r="D43" s="30" t="s">
-        <v>90</v>
-      </c>
-      <c r="E43" s="30"/>
+      <c r="C43" s="1"/>
+      <c r="D43" s="1"/>
+      <c r="E43" s="1"/>
     </row>
     <row r="44" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B44" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C44" s="39">
-        <f>market_capitalization / currentYear_equity</f>
-        <v>8.5378160491688046E-2</v>
-      </c>
-      <c r="D44" s="30" t="s">
-        <v>92</v>
+        <v>89</v>
+      </c>
+      <c r="C44" s="37">
+        <f>market_capitalization - (currentYear_equity / fx_usd_cny)</f>
+        <v>-766179.36175996368</v>
+      </c>
+      <c r="D44" s="57" t="s">
+        <v>352</v>
       </c>
       <c r="E44" s="30"/>
     </row>
     <row r="45" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B45" s="12" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C45" s="38">
+        <f>market_capitalization / (currentYear_equity / fx_usd_cny)</f>
+        <v>0.59727145953565286</v>
+      </c>
+      <c r="D45" s="57" t="s">
+        <v>353</v>
+      </c>
+      <c r="E45" s="30"/>
+    </row>
+    <row r="46" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B46" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C46" s="37">
         <f>currentYear_after_tax_operating_income-(cost_capital*startYear_total_capitalization)</f>
         <v>-1570336.21</v>
       </c>
-      <c r="D45" s="30" t="s">
+      <c r="D46" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="E46" s="30"/>
+    </row>
+    <row r="47" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B47" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C47" s="1"/>
+      <c r="D47" s="1"/>
+      <c r="E47" s="1"/>
+    </row>
+    <row r="48" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B48" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="E45" s="30"/>
-    </row>
-    <row r="46" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B46" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="C46" s="1"/>
-      <c r="D46" s="1"/>
-      <c r="E46" s="1"/>
-    </row>
-    <row r="47" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B47" s="12" t="s">
-        <v>96</v>
-      </c>
-      <c r="C47" s="40">
+      <c r="C48" s="39">
         <f>currentYear_after_tax_operating_income/startYear_total_assets</f>
         <v>1.0449377492937418E-2</v>
       </c>
-      <c r="D47" s="30" t="s">
-        <v>97</v>
-      </c>
-      <c r="E47" s="30"/>
-    </row>
-    <row r="48" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B48" s="12" t="s">
-        <v>98</v>
-      </c>
-      <c r="C48" s="40">
+      <c r="D48" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="E48" s="30"/>
+    </row>
+    <row r="49" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B49" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="C49" s="39">
         <f>currentYear_after_tax_operating_income/startYear_total_capitalization</f>
         <v>2.1008103757763935E-2</v>
       </c>
-      <c r="D48" s="30" t="s">
-        <v>99</v>
-      </c>
-      <c r="E48" s="30"/>
-    </row>
-    <row r="49" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B49" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="C49" s="40">
+      <c r="D49" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="E49" s="30"/>
+    </row>
+    <row r="50" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B50" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="C50" s="39">
         <f>INC_net/startYear_equity</f>
         <v>-1.5256961316200884E-2</v>
       </c>
-      <c r="D49" s="30" t="s">
-        <v>101</v>
-      </c>
-      <c r="E49" s="30"/>
-    </row>
-    <row r="50" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B50" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C50" s="40">
+      <c r="D50" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="E50" s="30"/>
+    </row>
+    <row r="51" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B51" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C51" s="39">
         <f>currentYear_after_tax_operating_income/avg_total_assets</f>
         <v>1.0345246860039986E-2</v>
       </c>
-      <c r="D50" s="30" t="s">
-        <v>103</v>
-      </c>
-      <c r="E50" s="30"/>
-    </row>
-    <row r="51" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B51" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="C51" s="40">
+      <c r="D51" s="30" t="s">
+        <v>101</v>
+      </c>
+      <c r="E51" s="30"/>
+    </row>
+    <row r="52" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B52" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="C52" s="39">
         <f>currentYear_after_tax_operating_income/avg_total_capitalization</f>
         <v>2.0721970888597039E-2</v>
       </c>
-      <c r="D51" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="E51" s="30"/>
-    </row>
-    <row r="52" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B52" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C52" s="40">
+      <c r="D52" s="30" t="s">
+        <v>103</v>
+      </c>
+      <c r="E52" s="30"/>
+    </row>
+    <row r="53" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B53" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="C53" s="39">
         <f>INC_net/avg_equity</f>
         <v>-1.5294035196601241E-2</v>
       </c>
-      <c r="D52" s="30" t="s">
+      <c r="D53" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="E53" s="30"/>
+    </row>
+    <row r="54" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B54" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C54" s="1"/>
+      <c r="D54" s="1"/>
+      <c r="E54" s="1"/>
+    </row>
+    <row r="55" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B55" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="E52" s="30"/>
-    </row>
-    <row r="53" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B53" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="C53" s="1"/>
-      <c r="D53" s="1"/>
-      <c r="E53" s="1"/>
-    </row>
-    <row r="54" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B54" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="C54" s="39">
+      <c r="C55" s="38">
         <f>INC_sales/startYear_total_assets</f>
         <v>0.59639394434395143</v>
       </c>
-      <c r="D54" s="30" t="s">
+      <c r="D55" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="E55" s="30" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="56" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B56" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="E54" s="30" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="55" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B55" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="C55" s="39">
+      <c r="C56" s="38">
         <f>INC_sales/startYear_receivables</f>
         <v>12.455081239406383</v>
       </c>
-      <c r="D55" s="30" t="s">
-        <v>113</v>
-      </c>
-      <c r="E55" s="30"/>
-    </row>
-    <row r="56" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B56" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="C56" s="41">
+      <c r="D56" s="30" t="s">
+        <v>111</v>
+      </c>
+      <c r="E56" s="30"/>
+    </row>
+    <row r="57" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B57" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="C57" s="40">
         <f>startYear_receivables/currentYear_daily_sales_average</f>
         <v>29.305308651475009</v>
       </c>
-      <c r="D56" s="30" t="s">
-        <v>115</v>
-      </c>
-      <c r="E56" s="30"/>
-    </row>
-    <row r="57" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B57" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="C57" s="39">
+      <c r="D57" s="30" t="s">
+        <v>113</v>
+      </c>
+      <c r="E57" s="30"/>
+    </row>
+    <row r="58" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B58" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="C58" s="38">
         <f>INC_cost_goods_sold/startYear_inventory</f>
         <v>55.418959245519886</v>
       </c>
-      <c r="D57" s="30" t="s">
-        <v>117</v>
-      </c>
-      <c r="E57" s="30"/>
-    </row>
-    <row r="58" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B58" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="C58" s="41">
+      <c r="D58" s="30" t="s">
+        <v>115</v>
+      </c>
+      <c r="E58" s="30"/>
+    </row>
+    <row r="59" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B59" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="C59" s="40">
         <f>startYear_inventory/currentYear_cost_goods_sold_daily</f>
         <v>6.5861936956080047</v>
       </c>
-      <c r="D58" s="30" t="s">
-        <v>119</v>
-      </c>
-      <c r="E58" s="30"/>
-    </row>
-    <row r="59" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B59" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="C59" s="40">
+      <c r="D59" s="30" t="s">
+        <v>117</v>
+      </c>
+      <c r="E59" s="30"/>
+    </row>
+    <row r="60" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B60" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="C60" s="39">
         <f>INC_net/INC_sales</f>
         <v>-7.47648518025891E-3</v>
       </c>
-      <c r="D59" s="30" t="s">
-        <v>121</v>
-      </c>
-      <c r="E59" s="30"/>
-    </row>
-    <row r="60" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B60" s="12" t="s">
-        <v>122</v>
-      </c>
-      <c r="C60" s="40">
+      <c r="D60" s="30" t="s">
+        <v>119</v>
+      </c>
+      <c r="E60" s="30"/>
+    </row>
+    <row r="61" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B61" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="C61" s="39">
         <f>currentYear_after_tax_operating_income/INC_sales</f>
         <v>1.7520931578928083E-2</v>
       </c>
-      <c r="D60" s="30" t="s">
+      <c r="D61" s="30" t="s">
+        <v>121</v>
+      </c>
+      <c r="E61" s="30" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="62" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B62" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="E60" s="30" t="s">
+      <c r="C62" s="1"/>
+      <c r="D62" s="1"/>
+      <c r="E62" s="1"/>
+    </row>
+    <row r="63" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B63" s="12" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="61" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B61" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="C61" s="1"/>
-      <c r="D61" s="1"/>
-      <c r="E61" s="1"/>
-    </row>
-    <row r="62" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B62" s="12" t="s">
-        <v>126</v>
-      </c>
-      <c r="C62" s="40">
+      <c r="C63" s="39">
         <f>currentYear_debt_long_term/(currentYear_debt_long_term+currentYear_equity)</f>
         <v>0.4309932342158424</v>
       </c>
-      <c r="D62" s="30" t="s">
-        <v>127</v>
-      </c>
-      <c r="E62" s="30"/>
-    </row>
-    <row r="63" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B63" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="C63" s="39">
+      <c r="D63" s="30" t="s">
+        <v>125</v>
+      </c>
+      <c r="E63" s="30"/>
+    </row>
+    <row r="64" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B64" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="C64" s="38">
         <f>currentYear_debt_long_term/currentYear_equity</f>
         <v>0.75744834707173214</v>
       </c>
-      <c r="D63" s="30" t="s">
-        <v>129</v>
-      </c>
-      <c r="E63" s="30"/>
-    </row>
-    <row r="64" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B64" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="C64" s="40">
+      <c r="D64" s="30" t="s">
+        <v>127</v>
+      </c>
+      <c r="E64" s="30"/>
+    </row>
+    <row r="65" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B65" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="C65" s="39">
         <f>currentYear_liabilities_total/currentYear_assets_total</f>
         <v>0.71490078507150601</v>
       </c>
-      <c r="D64" s="30" t="s">
-        <v>131</v>
-      </c>
-      <c r="E64" s="30"/>
-    </row>
-    <row r="65" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B65" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C65" s="39">
+      <c r="D65" s="30" t="s">
+        <v>129</v>
+      </c>
+      <c r="E65" s="30"/>
+    </row>
+    <row r="66" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B66" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C66" s="38">
         <f>INC_ebit/INC_interest_expense</f>
         <v>0.25210088652794144</v>
       </c>
-      <c r="D65" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="E65" s="30"/>
-    </row>
-    <row r="66" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B66" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="C66" s="39">
+      <c r="D66" s="30" t="s">
+        <v>131</v>
+      </c>
+      <c r="E66" s="30"/>
+    </row>
+    <row r="67" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B67" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="C67" s="38">
         <f>(INC_ebit+CF_depreciation_amortization)/INC_interest_expense</f>
         <v>14.834210260153736</v>
       </c>
-      <c r="D66" s="30" t="s">
-        <v>342</v>
-      </c>
-      <c r="E66" s="30" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="67" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B67" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="C67" s="42">
+      <c r="D67" s="30" t="s">
+        <v>340</v>
+      </c>
+      <c r="E67" s="30" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="68" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B68" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="C68" s="41">
         <f>INC_net/currentYear_after_tax_operating_income</f>
         <v>-0.42671733215662244</v>
       </c>
-      <c r="D67" s="30" t="s">
+      <c r="D68" s="30" t="s">
+        <v>134</v>
+      </c>
+      <c r="E68" s="30" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="69" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B69" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="E67" s="30" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="68" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B68" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="C68" s="39">
+      <c r="C69" s="38">
         <f>currentYear_assets_total/currentYear_equity</f>
         <v>3.5075508722491957</v>
       </c>
-      <c r="D68" s="30" t="s">
+      <c r="D69" s="30" t="s">
+        <v>137</v>
+      </c>
+      <c r="E69" s="30" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="70" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B70" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="E68" s="30" t="s">
+      <c r="C70" s="1"/>
+      <c r="D70" s="1"/>
+      <c r="E70" s="1"/>
+    </row>
+    <row r="71" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B71" s="12" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="69" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B69" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="C69" s="1"/>
-      <c r="D69" s="1"/>
-      <c r="E69" s="1"/>
-    </row>
-    <row r="70" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B70" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="C70" s="40">
+      <c r="C71" s="39">
         <f>currentYear_working_capital_net/currentYear_assets_total</f>
         <v>-0.25228308245184117</v>
       </c>
-      <c r="D70" s="30" t="s">
-        <v>143</v>
-      </c>
-      <c r="E70" s="30"/>
-    </row>
-    <row r="71" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B71" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="C71" s="39">
+      <c r="D71" s="30" t="s">
+        <v>141</v>
+      </c>
+      <c r="E71" s="30"/>
+    </row>
+    <row r="72" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B72" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="C72" s="38">
         <f>currentYear_assets_current/currentYear_liabilities_current</f>
         <v>0.46631403641595232</v>
       </c>
-      <c r="D71" s="30" t="s">
-        <v>145</v>
-      </c>
-      <c r="E71" s="30"/>
-    </row>
-    <row r="72" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B72" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="C72" s="39">
+      <c r="D72" s="30" t="s">
+        <v>143</v>
+      </c>
+      <c r="E72" s="30"/>
+    </row>
+    <row r="73" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B73" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="C73" s="38">
         <f>(currentYear_cash_marketable_securities+BAL_receivables_curr)/currentYear_liabilities_current</f>
         <v>0.31163489953712975</v>
       </c>
-      <c r="D72" s="30" t="s">
-        <v>147</v>
-      </c>
-      <c r="E72" s="30"/>
-    </row>
-    <row r="73" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B73" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="C73" s="39">
+      <c r="D73" s="30" t="s">
+        <v>145</v>
+      </c>
+      <c r="E73" s="30"/>
+    </row>
+    <row r="74" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B74" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="C74" s="38">
         <f>currentYear_cash_marketable_securities/currentYear_liabilities_current</f>
         <v>0.19731791468709797</v>
       </c>
-      <c r="D73" s="30" t="s">
+      <c r="D74" s="30" t="s">
+        <v>147</v>
+      </c>
+      <c r="E74" s="30"/>
+    </row>
+    <row r="75" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B75" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="C75" s="1"/>
+      <c r="D75" s="1"/>
+      <c r="E75" s="1"/>
+    </row>
+    <row r="76" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B76" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="E73" s="30"/>
-    </row>
-    <row r="74" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B74" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="C74" s="1"/>
-      <c r="D74" s="1"/>
-      <c r="E74" s="1"/>
-    </row>
-    <row r="75" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B75" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="C75" s="40">
+      <c r="C76" s="39">
         <f>RATIO_asset_turnover*RATIO_operating_profit_margin</f>
         <v>1.0449377492937416E-2</v>
       </c>
-      <c r="D75" s="30" t="s">
-        <v>152</v>
-      </c>
-      <c r="E75" s="30"/>
-      <c r="F75" s="44" t="str">
-        <f>IF(OR(C75="",C47=""),"",IF(ROUND(C75,6)=ROUND(C47,6),"✓ matches direct ROA","✗ differs by "&amp;TEXT(ABS(C75-C47),"0.00%")))</f>
+      <c r="D76" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="E76" s="30"/>
+      <c r="F76" s="43" t="str">
+        <f>IF(OR(C76="",C48=""),"",IF(ROUND(C76,6)=ROUND(C48,6),"✓ matches direct ROA","✗ differs by "&amp;TEXT(ABS(C76-C48),"0.00%")))</f>
         <v>✓ matches direct ROA</v>
       </c>
     </row>
-    <row r="76" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B76" s="12" t="s">
-        <v>153</v>
-      </c>
-      <c r="C76" s="40">
+    <row r="77" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B77" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="C77" s="39">
         <f>RATIO_leverage*RATIO_asset_turnover*RATIO_operating_profit_margin*RATIO_debt_burden</f>
         <v>-1.5639925517164466E-2</v>
       </c>
-      <c r="D76" s="30" t="s">
-        <v>154</v>
-      </c>
-      <c r="E76" s="30"/>
+      <c r="D77" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="E77" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B21:E21"/>
-    <mergeCell ref="B35:E35"/>
-    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B15:E15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4212,228 +4367,228 @@
   <sheetData>
     <row r="2" spans="2:4" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="14" t="s">
+        <v>280</v>
+      </c>
+      <c r="C2" s="14"/>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B4" s="42" t="s">
+        <v>281</v>
+      </c>
+      <c r="C4" s="42" t="s">
+        <v>318</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>282</v>
       </c>
-      <c r="C2" s="14"/>
-    </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B4" s="43" t="s">
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B5" s="42" t="s">
         <v>283</v>
       </c>
-      <c r="C4" s="43" t="s">
+      <c r="C5" s="42" t="s">
+        <v>319</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B6" s="42" t="s">
+        <v>285</v>
+      </c>
+      <c r="C6" s="42" t="s">
         <v>320</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B5" s="43" t="s">
-        <v>285</v>
-      </c>
-      <c r="C5" s="43" t="s">
+      <c r="D6" s="4" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B7" s="42" t="s">
+        <v>287</v>
+      </c>
+      <c r="C7" s="42" t="s">
         <v>321</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B6" s="43" t="s">
-        <v>287</v>
-      </c>
-      <c r="C6" s="43" t="s">
+      <c r="D7" s="4" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B8" s="42" t="s">
+        <v>289</v>
+      </c>
+      <c r="C8" s="42" t="s">
         <v>322</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B7" s="43" t="s">
-        <v>289</v>
-      </c>
-      <c r="C7" s="43" t="s">
+    <row r="9" spans="2:4" ht="75" x14ac:dyDescent="0.2">
+      <c r="B9" s="42" t="s">
+        <v>342</v>
+      </c>
+      <c r="C9" s="45" t="s">
+        <v>343</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" ht="30" x14ac:dyDescent="0.2">
+      <c r="B10" s="42" t="s">
+        <v>345</v>
+      </c>
+      <c r="C10" s="42" t="s">
+        <v>346</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B11" s="42" t="s">
+        <v>290</v>
+      </c>
+      <c r="C11" s="42" t="s">
         <v>323</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B8" s="43" t="s">
+      <c r="D11" s="4" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B12" s="42" t="s">
         <v>291</v>
       </c>
-      <c r="C8" s="43" t="s">
+      <c r="C12" s="42" t="s">
         <v>324</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="9" spans="2:4" ht="75" x14ac:dyDescent="0.2">
-      <c r="B9" s="43" t="s">
-        <v>344</v>
-      </c>
-      <c r="C9" s="46" t="s">
-        <v>345</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="10" spans="2:4" ht="30" x14ac:dyDescent="0.2">
-      <c r="B10" s="43" t="s">
-        <v>347</v>
-      </c>
-      <c r="C10" s="43" t="s">
-        <v>348</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B11" s="43" t="s">
+      <c r="D12" s="4" t="s">
         <v>292</v>
       </c>
-      <c r="C11" s="43" t="s">
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B13" s="42" t="s">
+        <v>293</v>
+      </c>
+      <c r="C13" s="42" t="s">
         <v>325</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B12" s="43" t="s">
-        <v>293</v>
-      </c>
-      <c r="C12" s="43" t="s">
+      <c r="D13" s="4" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B14" s="42" t="s">
+        <v>295</v>
+      </c>
+      <c r="C14" s="42" t="s">
         <v>326</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B13" s="43" t="s">
-        <v>295</v>
-      </c>
-      <c r="C13" s="43" t="s">
+      <c r="D14" s="4" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B15" s="42" t="s">
+        <v>297</v>
+      </c>
+      <c r="C15" s="42" t="s">
         <v>327</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B14" s="43" t="s">
-        <v>297</v>
-      </c>
-      <c r="C14" s="43" t="s">
+      <c r="D15" s="4" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B17" s="42" t="s">
+        <v>299</v>
+      </c>
+      <c r="C17" s="42"/>
+      <c r="D17" s="4" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="42" t="s">
+        <v>301</v>
+      </c>
+      <c r="C18" s="42" t="s">
         <v>328</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B15" s="43" t="s">
-        <v>299</v>
-      </c>
-      <c r="C15" s="43" t="s">
+      <c r="D18" s="4" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="42" t="s">
+        <v>303</v>
+      </c>
+      <c r="C19" s="45" t="s">
+        <v>330</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="42" t="s">
+        <v>305</v>
+      </c>
+      <c r="C20" s="42" t="s">
         <v>329</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B17" s="43" t="s">
-        <v>301</v>
-      </c>
-      <c r="C17" s="43"/>
-      <c r="D17" s="4" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="43" t="s">
-        <v>303</v>
-      </c>
-      <c r="C18" s="43" t="s">
-        <v>330</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="19" spans="2:4" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="43" t="s">
-        <v>305</v>
-      </c>
-      <c r="C19" s="46" t="s">
-        <v>332</v>
-      </c>
-      <c r="D19" s="4" t="s">
+      <c r="D20" s="4" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="20" spans="2:4" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="43" t="s">
+    <row r="21" spans="2:4" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="42" t="s">
         <v>307</v>
       </c>
-      <c r="C20" s="43" t="s">
-        <v>331</v>
-      </c>
-      <c r="D20" s="4" t="s">
+      <c r="C21" s="42" t="s">
+        <v>329</v>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="21" spans="2:4" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="43" t="s">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B23" s="42" t="s">
         <v>309</v>
       </c>
-      <c r="C21" s="43" t="s">
-        <v>331</v>
-      </c>
-      <c r="D21" s="4" t="s">
+      <c r="C23" s="42"/>
+    </row>
+    <row r="24" spans="2:4" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="42" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B23" s="43" t="s">
+      <c r="C24" s="42"/>
+      <c r="D24" s="4" t="s">
         <v>311</v>
       </c>
-      <c r="C23" s="43"/>
-    </row>
-    <row r="24" spans="2:4" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="43" t="s">
+    </row>
+    <row r="25" spans="2:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="42" t="s">
         <v>312</v>
       </c>
-      <c r="C24" s="43"/>
-      <c r="D24" s="4" t="s">
+      <c r="C25" s="42"/>
+      <c r="D25" s="4" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="25" spans="2:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="43" t="s">
-        <v>314</v>
-      </c>
-      <c r="C25" s="43"/>
-      <c r="D25" s="4" t="s">
-        <v>315</v>
-      </c>
-    </row>
     <row r="26" spans="2:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="43" t="s">
+      <c r="B26" s="42" t="s">
+        <v>333</v>
+      </c>
+      <c r="C26" s="42" t="s">
+        <v>334</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>335</v>
-      </c>
-      <c r="C26" s="43" t="s">
-        <v>336</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
writing final analysis, llm raw and edit finacials
</commit_message>
<xml_diff>
--- a/models/builds/2026-05-14-luong-iqiyi-financials.xlsx
+++ b/models/builds/2026-05-14-luong-iqiyi-financials.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luongduyphuong/Documents/GitHub/Corporate-Finance/models/builds/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62DD2FB6-05A4-304A-893A-DECC8D95A672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D36F9D0B-1AFE-0A4D-9FD7-64C26FB94EE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -2004,6 +2004,14 @@
     </xf>
     <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="172" fontId="9" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2012,14 +2020,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="172" fontId="9" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2383,32 +2383,32 @@
       <c r="C2" s="1"/>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B4" s="50" t="s">
+      <c r="B4" s="56" t="s">
         <v>153</v>
       </c>
-      <c r="C4" s="49"/>
+      <c r="C4" s="55"/>
     </row>
     <row r="5" spans="2:3" ht="26" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="53" t="s">
+      <c r="B5" s="59" t="s">
         <v>154</v>
       </c>
-      <c r="C5" s="49"/>
+      <c r="C5" s="55"/>
     </row>
     <row r="6" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="51" t="s">
+      <c r="B6" s="57" t="s">
         <v>155</v>
       </c>
-      <c r="C6" s="49"/>
+      <c r="C6" s="55"/>
     </row>
     <row r="7" spans="2:3" ht="4" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
     </row>
     <row r="9" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="52" t="s">
+      <c r="B9" s="58" t="s">
         <v>156</v>
       </c>
-      <c r="C9" s="49"/>
+      <c r="C9" s="55"/>
     </row>
     <row r="10" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="3" t="s">
@@ -2459,10 +2459,10 @@
       </c>
     </row>
     <row r="17" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="52" t="s">
+      <c r="B17" s="58" t="s">
         <v>169</v>
       </c>
-      <c r="C17" s="49"/>
+      <c r="C17" s="55"/>
     </row>
     <row r="18" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="5" t="s">
@@ -2505,10 +2505,10 @@
       </c>
     </row>
     <row r="24" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="52" t="s">
+      <c r="B24" s="58" t="s">
         <v>180</v>
       </c>
-      <c r="C24" s="49"/>
+      <c r="C24" s="55"/>
     </row>
     <row r="25" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="5" t="s">
@@ -2583,10 +2583,10 @@
       </c>
     </row>
     <row r="36" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="52" t="s">
+      <c r="B36" s="58" t="s">
         <v>198</v>
       </c>
-      <c r="C36" s="49"/>
+      <c r="C36" s="55"/>
     </row>
     <row r="37" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="12" t="s">
@@ -2605,10 +2605,10 @@
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B41" s="54" t="s">
+      <c r="B41" s="60" t="s">
         <v>203</v>
       </c>
-      <c r="C41" s="49"/>
+      <c r="C41" s="55"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -3535,7 +3535,7 @@
       <c r="B12" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="56">
+      <c r="C12" s="49">
         <f>share_price*shares_outstanding</f>
         <v>1136291.6199999999</v>
       </c>
@@ -3547,29 +3547,29 @@
       </c>
     </row>
     <row r="13" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="55" t="s">
+      <c r="B13" s="48" t="s">
         <v>349</v>
       </c>
-      <c r="C13" s="60">
+      <c r="C13" s="53">
         <v>6.9955999999999996</v>
       </c>
-      <c r="D13" s="58" t="s">
+      <c r="D13" s="51" t="s">
         <v>350</v>
       </c>
-      <c r="E13" s="57" t="s">
+      <c r="E13" s="50" t="s">
         <v>348</v>
       </c>
-      <c r="F13" s="59" t="s">
+      <c r="F13" s="52" t="s">
         <v>351</v>
       </c>
     </row>
     <row r="15" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="48" t="s">
+      <c r="B15" s="54" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="49"/>
-      <c r="D15" s="49"/>
-      <c r="E15" s="49"/>
+      <c r="C15" s="55"/>
+      <c r="D15" s="55"/>
+      <c r="E15" s="55"/>
     </row>
     <row r="16" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="12" t="s">
@@ -3647,12 +3647,12 @@
       </c>
     </row>
     <row r="22" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="48" t="s">
+      <c r="B22" s="54" t="s">
         <v>37</v>
       </c>
-      <c r="C22" s="49"/>
-      <c r="D22" s="49"/>
-      <c r="E22" s="49"/>
+      <c r="C22" s="55"/>
+      <c r="D22" s="55"/>
+      <c r="E22" s="55"/>
     </row>
     <row r="23" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="12" t="s">
@@ -3835,12 +3835,12 @@
       </c>
     </row>
     <row r="36" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="48" t="s">
+      <c r="B36" s="54" t="s">
         <v>74</v>
       </c>
-      <c r="C36" s="49"/>
-      <c r="D36" s="49"/>
-      <c r="E36" s="49"/>
+      <c r="C36" s="55"/>
+      <c r="D36" s="55"/>
+      <c r="E36" s="55"/>
     </row>
     <row r="37" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="12" t="s">
@@ -3920,7 +3920,7 @@
         <f>market_capitalization - (currentYear_equity / fx_usd_cny)</f>
         <v>-766179.36175996368</v>
       </c>
-      <c r="D44" s="57" t="s">
+      <c r="D44" s="50" t="s">
         <v>352</v>
       </c>
       <c r="E44" s="30"/>
@@ -3933,7 +3933,7 @@
         <f>market_capitalization / (currentYear_equity / fx_usd_cny)</f>
         <v>0.59727145953565286</v>
       </c>
-      <c r="D45" s="57" t="s">
+      <c r="D45" s="50" t="s">
         <v>353</v>
       </c>
       <c r="E45" s="30"/>

</xml_diff>